<commit_message>
Self-host ambient videos under /media-da/videos
The importer now points mp4 links at the site's own copies, and
video.js accepts a site-relative video path in the link text.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-solutions.report.xlsx
+++ b/tools/importer/reports/import-solutions.report.xlsx
@@ -52,7 +52,7 @@
     <t>solutions</t>
   </si>
   <si>
-    <t>2026-10-19T20:49:45.912Z</t>
+    <t>2026-10-19T21:49:04.571Z</t>
   </si>
   <si>
     <t>Content Supply Chain Solution | Adobe AI Marketing Workflows</t>
@@ -73,7 +73,7 @@
     <t>content-supply-chain</t>
   </si>
   <si>
-    <t>2026-10-19T10:20:21.912Z</t>
+    <t>2026-10-19T20:50:01.299Z</t>
   </si>
   <si>
     <t>Asset Management for Enterprise | Adobe Content Supply Chain</t>
@@ -91,7 +91,7 @@
     <t>solutions/content-supply-chain/content-insights</t>
   </si>
   <si>
-    <t>2026-10-19T10:20:32.962Z</t>
+    <t>2026-10-19T20:50:13.015Z</t>
   </si>
   <si>
     <t>Content Reporting &amp; Insights | Adobe Content Supply Chain</t>
@@ -109,7 +109,7 @@
     <t>solutions/content-supply-chain/marketer-led-creation</t>
   </si>
   <si>
-    <t>2026-10-19T10:20:45.074Z</t>
+    <t>2026-10-19T20:50:24.016Z</t>
   </si>
   <si>
     <t>Marketer-led Content Creation | Adobe Content Supply Chain</t>
@@ -127,7 +127,7 @@
     <t>solutions/content-supply-chain/rebuild-creative-foundations</t>
   </si>
   <si>
-    <t>2026-10-19T10:20:57.243Z</t>
+    <t>2026-10-19T20:50:35.721Z</t>
   </si>
   <si>
     <t>Rebuild Creative Foundations | Adobe Content Supply Chain</t>
@@ -145,7 +145,7 @@
     <t>solutions/content-supply-chain/scaled-content-production</t>
   </si>
   <si>
-    <t>2026-10-19T10:21:07.174Z</t>
+    <t>2026-10-19T20:50:50.018Z</t>
   </si>
   <si>
     <t>Scaled Content Production | Adobe Content Supply Chain</t>
@@ -163,7 +163,7 @@
     <t>solutions/content-supply-chain/workflow-planning</t>
   </si>
   <si>
-    <t>2026-10-19T10:21:18.993Z</t>
+    <t>2026-10-19T20:51:01.291Z</t>
   </si>
   <si>
     <t>Content Supply Chain Workflow, Planning, &amp; Metadata | Adobe for Business</t>

</xml_diff>